<commit_message>
Upload de arquivos para verificar erro do make volumes no MAC
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/bancos/SISOR/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\SEPLAG\2022\SPLOR\DCPPN\LeiOrcamentariaAnual\LOA\bancos\SISOR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72D73F02-82B8-4576-B7B8-54DEC71DE37A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{17E7E226-1BB7-442E-A82D-B32F9EC6D3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="150" windowWidth="21600" windowHeight="11145"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="10890"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DETALHAMENTO_OBRAS" sheetId="1" r:id="rId1"/>
@@ -2079,7 +2079,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 10092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/bancos/SISOR/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -7142,7 +7142,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>REDIMENSIONAMENTO DE REDE ELÉTRICA (NRPMSO'S) - Garantir a segurança elétrica para implementação de novos equipamentos</t>
+          <t>REDIMENSIONAMENTO DE REDE ELÉTRICA (NRPMSO`S) - Garantir a segurança elétrica para implementação de novos equipamentos</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -13964,7 +13964,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>CONSERVAÇÃO DA MALHA VIÁRIA DAS 40ª URG'S</t>
+          <t>CONSERVAÇÃO DA MALHA VIÁRIA DAS 40ª URG`S</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">

</xml_diff>